<commit_message>
Publish autonomous monthly urinary evidence update
</commit_message>
<xml_diff>
--- a/summary/no/exposures_meta_analysis_aggressive_prostate_cancer_combined.xlsx
+++ b/summary/no/exposures_meta_analysis_aggressive_prostate_cancer_combined.xlsx
@@ -779,7 +779,7 @@
         <v>76.5</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.2832792558734613</v>
+        <v>0.2832792558734611</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>114280</v>
@@ -814,7 +814,7 @@
         <v>89.40000000000001</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0.8385914121835611</v>
+        <v>0.8385914121835617</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>123475</v>
@@ -915,7 +915,7 @@
         <v>81.90000000000001</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.2069198638695531</v>
+        <v>0.2069198638695532</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>45247</v>
@@ -1279,7 +1279,7 @@
         <v>80</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.4695295847551802</v>
+        <v>0.4695295847551806</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>166503</v>
@@ -1448,7 +1448,7 @@
         <v>0</v>
       </c>
       <c r="I31" s="5" t="n">
-        <v>0.256016891196605</v>
+        <v>0.2560168911966049</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>101424</v>
@@ -1516,7 +1516,7 @@
         <v>86</v>
       </c>
       <c r="I33" s="5" t="n">
-        <v>0.01966497897827826</v>
+        <v>0.01966497897827823</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>383989</v>

</xml_diff>

<commit_message>
Add opt-in Europe PMC preprint recovery and navy provenance
</commit_message>
<xml_diff>
--- a/summary/no/exposures_meta_analysis_aggressive_prostate_cancer_combined.xlsx
+++ b/summary/no/exposures_meta_analysis_aggressive_prostate_cancer_combined.xlsx
@@ -24,13 +24,16 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -50,7 +53,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -58,13 +61,22 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -453,57 +465,57 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Exposure</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>number studies</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Pooled RR</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>lower CI RR</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>upper CI RR</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>lower PI RR</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>upper PI RR</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>I^2 (%)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>eggers p-value</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>total N</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>total Cases</t>
         </is>
@@ -515,28 +527,28 @@
           <t>magnesium</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" s="3" t="n">
+      <c r="B2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="4" t="n">
         <v>0.26</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D2" s="4" t="n">
         <v>0.09</v>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="E2" s="4" t="n">
         <v>0.85</v>
       </c>
-      <c r="F2" s="3" t="inlineStr"/>
-      <c r="G2" s="3" t="inlineStr"/>
-      <c r="H2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" s="5" t="inlineStr"/>
-      <c r="J2" s="2" t="n">
+      <c r="F2" s="4" t="inlineStr"/>
+      <c r="G2" s="4" t="inlineStr"/>
+      <c r="H2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="6" t="inlineStr"/>
+      <c r="J2" s="3" t="n">
         <v>261</v>
       </c>
-      <c r="K2" s="2" t="n">
+      <c r="K2" s="3" t="n">
         <v>98</v>
       </c>
     </row>
@@ -546,28 +558,28 @@
           <t>vitamin_k2</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" s="3" t="n">
+      <c r="B3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="4" t="n">
         <v>0.37</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D3" s="4" t="n">
         <v>0.16</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="E3" s="4" t="n">
         <v>0.88</v>
       </c>
-      <c r="F3" s="3" t="inlineStr"/>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="5" t="inlineStr"/>
-      <c r="J3" s="2" t="n">
+      <c r="F3" s="4" t="inlineStr"/>
+      <c r="G3" s="4" t="inlineStr"/>
+      <c r="H3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="6" t="inlineStr"/>
+      <c r="J3" s="3" t="n">
         <v>11319</v>
       </c>
-      <c r="K3" s="2" t="n">
+      <c r="K3" s="3" t="n">
         <v>113</v>
       </c>
     </row>
@@ -577,28 +589,28 @@
           <t>insoluble_dietary_fiber_intake</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" s="3" t="n">
+      <c r="B4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="4" t="n">
         <v>0.46</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="D4" s="4" t="n">
         <v>0.22</v>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="E4" s="4" t="n">
         <v>0.93</v>
       </c>
-      <c r="F4" s="3" t="inlineStr"/>
-      <c r="G4" s="3" t="inlineStr"/>
-      <c r="H4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="5" t="inlineStr"/>
-      <c r="J4" s="2" t="n">
+      <c r="F4" s="4" t="inlineStr"/>
+      <c r="G4" s="4" t="inlineStr"/>
+      <c r="H4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="6" t="inlineStr"/>
+      <c r="J4" s="3" t="n">
         <v>43435</v>
       </c>
-      <c r="K4" s="2" t="inlineStr"/>
+      <c r="K4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -606,28 +618,28 @@
           <t>green_tea</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" s="3" t="n">
+      <c r="B5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="4" t="n">
         <v>0.52</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D5" s="4" t="n">
         <v>0.28</v>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="E5" s="4" t="n">
         <v>0.96</v>
       </c>
-      <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="3" t="inlineStr"/>
-      <c r="H5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="5" t="inlineStr"/>
-      <c r="J5" s="2" t="n">
+      <c r="F5" s="4" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="6" t="inlineStr"/>
+      <c r="J5" s="3" t="n">
         <v>49920</v>
       </c>
-      <c r="K5" s="2" t="n">
+      <c r="K5" s="3" t="n">
         <v>114</v>
       </c>
     </row>
@@ -637,28 +649,28 @@
           <t>tea</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" s="3" t="n">
+      <c r="B6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="4" t="n">
         <v>0.52</v>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="D6" s="4" t="n">
         <v>0.28</v>
       </c>
-      <c r="E6" s="3" t="n">
+      <c r="E6" s="4" t="n">
         <v>0.96</v>
       </c>
-      <c r="F6" s="3" t="inlineStr"/>
-      <c r="G6" s="3" t="inlineStr"/>
-      <c r="H6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="5" t="inlineStr"/>
-      <c r="J6" s="2" t="n">
+      <c r="F6" s="4" t="inlineStr"/>
+      <c r="G6" s="4" t="inlineStr"/>
+      <c r="H6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="6" t="inlineStr"/>
+      <c r="J6" s="3" t="n">
         <v>49920</v>
       </c>
-      <c r="K6" s="2" t="n">
+      <c r="K6" s="3" t="n">
         <v>114</v>
       </c>
     </row>
@@ -668,28 +680,28 @@
           <t>inositol</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" s="3" t="n">
+      <c r="B7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="4" t="n">
         <v>0.5600000000000001</v>
       </c>
-      <c r="D7" s="3" t="n">
+      <c r="D7" s="4" t="n">
         <v>0.39</v>
       </c>
-      <c r="E7" s="3" t="n">
+      <c r="E7" s="4" t="n">
         <v>0.8100000000000001</v>
       </c>
-      <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="3" t="inlineStr"/>
-      <c r="H7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="5" t="inlineStr"/>
-      <c r="J7" s="2" t="n">
+      <c r="F7" s="4" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr"/>
+      <c r="H7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="6" t="inlineStr"/>
+      <c r="J7" s="3" t="n">
         <v>400</v>
       </c>
-      <c r="K7" s="2" t="n">
+      <c r="K7" s="3" t="n">
         <v>100</v>
       </c>
     </row>
@@ -699,28 +711,28 @@
           <t>lycopene</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B8" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C8" s="4" t="n">
         <v>0.58</v>
       </c>
-      <c r="D8" s="3" t="n">
+      <c r="D8" s="4" t="n">
         <v>0.39</v>
       </c>
-      <c r="E8" s="3" t="n">
+      <c r="E8" s="4" t="n">
         <v>0.87</v>
       </c>
-      <c r="F8" s="3" t="inlineStr"/>
-      <c r="G8" s="3" t="inlineStr"/>
-      <c r="H8" s="4" t="n">
+      <c r="F8" s="4" t="inlineStr"/>
+      <c r="G8" s="4" t="inlineStr"/>
+      <c r="H8" s="5" t="n">
         <v>22.3</v>
       </c>
-      <c r="I8" s="5" t="inlineStr"/>
-      <c r="J8" s="2" t="n">
+      <c r="I8" s="6" t="inlineStr"/>
+      <c r="J8" s="3" t="n">
         <v>166781</v>
       </c>
-      <c r="K8" s="2" t="inlineStr"/>
+      <c r="K8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -728,28 +740,28 @@
           <t>beta_carotene</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" s="3" t="n">
+      <c r="B9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="4" t="n">
         <v>0.6</v>
       </c>
-      <c r="D9" s="3" t="n">
+      <c r="D9" s="4" t="n">
         <v>0.3</v>
       </c>
-      <c r="E9" s="3" t="n">
+      <c r="E9" s="4" t="n">
         <v>1.6</v>
       </c>
-      <c r="F9" s="3" t="inlineStr"/>
-      <c r="G9" s="3" t="inlineStr"/>
-      <c r="H9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="5" t="inlineStr"/>
-      <c r="J9" s="2" t="n">
+      <c r="F9" s="4" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="3" t="n">
         <v>1037</v>
       </c>
-      <c r="K9" s="2" t="inlineStr"/>
+      <c r="K9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -757,34 +769,34 @@
           <t>vitamin_e</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="C10" s="3" t="n">
+      <c r="C10" s="4" t="n">
         <v>0.64</v>
       </c>
-      <c r="D10" s="3" t="n">
+      <c r="D10" s="4" t="n">
         <v>0.4</v>
       </c>
-      <c r="E10" s="3" t="n">
+      <c r="E10" s="4" t="n">
         <v>1.04</v>
       </c>
-      <c r="F10" s="3" t="n">
+      <c r="F10" s="4" t="n">
         <v>0.08</v>
       </c>
-      <c r="G10" s="3" t="n">
+      <c r="G10" s="4" t="n">
         <v>5.21</v>
       </c>
-      <c r="H10" s="4" t="n">
+      <c r="H10" s="5" t="n">
         <v>76.5</v>
       </c>
-      <c r="I10" s="5" t="n">
-        <v>0.2832792558734611</v>
-      </c>
-      <c r="J10" s="2" t="n">
+      <c r="I10" s="6" t="n">
+        <v>0.2832792558734609</v>
+      </c>
+      <c r="J10" s="3" t="n">
         <v>114280</v>
       </c>
-      <c r="K10" s="2" t="inlineStr"/>
+      <c r="K10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -792,34 +804,34 @@
           <t>selenium</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B11" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="C11" s="3" t="n">
+      <c r="C11" s="4" t="n">
         <v>0.65</v>
       </c>
-      <c r="D11" s="3" t="n">
+      <c r="D11" s="4" t="n">
         <v>0.37</v>
       </c>
-      <c r="E11" s="3" t="n">
+      <c r="E11" s="4" t="n">
         <v>1.12</v>
       </c>
-      <c r="F11" s="3" t="n">
+      <c r="F11" s="4" t="n">
         <v>0.09</v>
       </c>
-      <c r="G11" s="3" t="n">
+      <c r="G11" s="4" t="n">
         <v>4.9</v>
       </c>
-      <c r="H11" s="4" t="n">
+      <c r="H11" s="5" t="n">
         <v>89.40000000000001</v>
       </c>
-      <c r="I11" s="5" t="n">
+      <c r="I11" s="6" t="n">
         <v>0.8385914121835617</v>
       </c>
-      <c r="J11" s="2" t="n">
+      <c r="J11" s="3" t="n">
         <v>123475</v>
       </c>
-      <c r="K11" s="2" t="inlineStr"/>
+      <c r="K11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -827,34 +839,34 @@
           <t>tomato</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B12" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C12" s="3" t="n">
+      <c r="C12" s="4" t="n">
         <v>0.7</v>
       </c>
-      <c r="D12" s="3" t="n">
+      <c r="D12" s="4" t="n">
         <v>0.54</v>
       </c>
-      <c r="E12" s="3" t="n">
+      <c r="E12" s="4" t="n">
         <v>0.9</v>
       </c>
-      <c r="F12" s="3" t="n">
+      <c r="F12" s="4" t="n">
         <v>0.14</v>
       </c>
-      <c r="G12" s="3" t="n">
+      <c r="G12" s="4" t="n">
         <v>3.54</v>
       </c>
-      <c r="H12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="5" t="n">
+      <c r="H12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="6" t="n">
         <v>0.1511955352792509</v>
       </c>
-      <c r="J12" s="2" t="n">
+      <c r="J12" s="3" t="n">
         <v>124620</v>
       </c>
-      <c r="K12" s="2" t="inlineStr"/>
+      <c r="K12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -862,28 +874,28 @@
           <t>legumes</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C13" s="3" t="n">
+      <c r="B13" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="4" t="n">
         <v>0.74</v>
       </c>
-      <c r="D13" s="3" t="n">
+      <c r="D13" s="4" t="n">
         <v>0.61</v>
       </c>
-      <c r="E13" s="3" t="n">
+      <c r="E13" s="4" t="n">
         <v>0.9</v>
       </c>
-      <c r="F13" s="3" t="inlineStr"/>
-      <c r="G13" s="3" t="inlineStr"/>
-      <c r="H13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="5" t="inlineStr"/>
-      <c r="J13" s="2" t="n">
+      <c r="F13" s="4" t="inlineStr"/>
+      <c r="G13" s="4" t="inlineStr"/>
+      <c r="H13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="6" t="inlineStr"/>
+      <c r="J13" s="3" t="n">
         <v>82483</v>
       </c>
-      <c r="K13" s="2" t="n">
+      <c r="K13" s="3" t="n">
         <v>1278</v>
       </c>
     </row>
@@ -893,34 +905,34 @@
           <t>vitamin_d</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B14" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="C14" s="3" t="n">
+      <c r="C14" s="4" t="n">
         <v>0.74</v>
       </c>
-      <c r="D14" s="3" t="n">
+      <c r="D14" s="4" t="n">
         <v>0.51</v>
       </c>
-      <c r="E14" s="3" t="n">
+      <c r="E14" s="4" t="n">
         <v>1.08</v>
       </c>
-      <c r="F14" s="3" t="n">
+      <c r="F14" s="4" t="n">
         <v>0.21</v>
       </c>
-      <c r="G14" s="3" t="n">
+      <c r="G14" s="4" t="n">
         <v>2.56</v>
       </c>
-      <c r="H14" s="4" t="n">
+      <c r="H14" s="5" t="n">
         <v>81.90000000000001</v>
       </c>
-      <c r="I14" s="5" t="n">
-        <v>0.2069198638695532</v>
-      </c>
-      <c r="J14" s="2" t="n">
+      <c r="I14" s="6" t="n">
+        <v>0.2069198638695529</v>
+      </c>
+      <c r="J14" s="3" t="n">
         <v>45247</v>
       </c>
-      <c r="K14" s="2" t="inlineStr"/>
+      <c r="K14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -928,28 +940,28 @@
           <t>folic_acid</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C15" s="3" t="n">
+      <c r="B15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="4" t="n">
         <v>0.78</v>
       </c>
-      <c r="D15" s="3" t="n">
+      <c r="D15" s="4" t="n">
         <v>0.53</v>
       </c>
-      <c r="E15" s="3" t="n">
+      <c r="E15" s="4" t="n">
         <v>1.15</v>
       </c>
-      <c r="F15" s="3" t="inlineStr"/>
-      <c r="G15" s="3" t="inlineStr"/>
-      <c r="H15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="5" t="inlineStr"/>
-      <c r="J15" s="2" t="n">
+      <c r="F15" s="4" t="inlineStr"/>
+      <c r="G15" s="4" t="inlineStr"/>
+      <c r="H15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="6" t="inlineStr"/>
+      <c r="J15" s="3" t="n">
         <v>65836</v>
       </c>
-      <c r="K15" s="2" t="inlineStr"/>
+      <c r="K15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -957,28 +969,28 @@
           <t>eicosapentaenoic_acid</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C16" s="3" t="n">
+      <c r="B16" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="D16" s="3" t="n">
+      <c r="D16" s="4" t="n">
         <v>0.64</v>
       </c>
-      <c r="E16" s="3" t="n">
+      <c r="E16" s="4" t="n">
         <v>1.04</v>
       </c>
-      <c r="F16" s="3" t="inlineStr"/>
-      <c r="G16" s="3" t="inlineStr"/>
-      <c r="H16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="5" t="inlineStr"/>
-      <c r="J16" s="2" t="n">
+      <c r="F16" s="4" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr"/>
+      <c r="H16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="6" t="inlineStr"/>
+      <c r="J16" s="3" t="n">
         <v>288268</v>
       </c>
-      <c r="K16" s="2" t="n">
+      <c r="K16" s="3" t="n">
         <v>725</v>
       </c>
     </row>
@@ -988,28 +1000,28 @@
           <t>zinc</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n">
+      <c r="B17" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C17" s="3" t="n">
+      <c r="C17" s="4" t="n">
         <v>0.84</v>
       </c>
-      <c r="D17" s="3" t="n">
+      <c r="D17" s="4" t="n">
         <v>0.17</v>
       </c>
-      <c r="E17" s="3" t="n">
+      <c r="E17" s="4" t="n">
         <v>4.29</v>
       </c>
-      <c r="F17" s="3" t="inlineStr"/>
-      <c r="G17" s="3" t="inlineStr"/>
-      <c r="H17" s="4" t="n">
+      <c r="F17" s="4" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr"/>
+      <c r="H17" s="5" t="n">
         <v>87.8</v>
       </c>
-      <c r="I17" s="5" t="inlineStr"/>
-      <c r="J17" s="2" t="n">
+      <c r="I17" s="6" t="inlineStr"/>
+      <c r="J17" s="3" t="n">
         <v>82482</v>
       </c>
-      <c r="K17" s="2" t="inlineStr"/>
+      <c r="K17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1017,28 +1029,28 @@
           <t>dash_diet</t>
         </is>
       </c>
-      <c r="B18" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C18" s="3" t="n">
+      <c r="B18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="4" t="n">
         <v>0.86</v>
       </c>
-      <c r="D18" s="3" t="n">
+      <c r="D18" s="4" t="n">
         <v>0.77</v>
       </c>
-      <c r="E18" s="3" t="n">
+      <c r="E18" s="4" t="n">
         <v>0.98</v>
       </c>
-      <c r="F18" s="3" t="inlineStr"/>
-      <c r="G18" s="3" t="inlineStr"/>
-      <c r="H18" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="5" t="inlineStr"/>
-      <c r="J18" s="2" t="n">
+      <c r="F18" s="4" t="inlineStr"/>
+      <c r="G18" s="4" t="inlineStr"/>
+      <c r="H18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="6" t="inlineStr"/>
+      <c r="J18" s="3" t="n">
         <v>79930</v>
       </c>
-      <c r="K18" s="2" t="inlineStr"/>
+      <c r="K18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1046,28 +1058,28 @@
           <t>total_dietary_fiber_intake</t>
         </is>
       </c>
-      <c r="B19" s="2" t="n">
+      <c r="B19" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C19" s="3" t="n">
+      <c r="C19" s="4" t="n">
         <v>0.86</v>
       </c>
-      <c r="D19" s="3" t="n">
+      <c r="D19" s="4" t="n">
         <v>0.63</v>
       </c>
-      <c r="E19" s="3" t="n">
+      <c r="E19" s="4" t="n">
         <v>1.17</v>
       </c>
-      <c r="F19" s="3" t="inlineStr"/>
-      <c r="G19" s="3" t="inlineStr"/>
-      <c r="H19" s="4" t="n">
+      <c r="F19" s="4" t="inlineStr"/>
+      <c r="G19" s="4" t="inlineStr"/>
+      <c r="H19" s="5" t="n">
         <v>51.2</v>
       </c>
-      <c r="I19" s="5" t="inlineStr"/>
-      <c r="J19" s="2" t="n">
+      <c r="I19" s="6" t="inlineStr"/>
+      <c r="J19" s="3" t="n">
         <v>885584</v>
       </c>
-      <c r="K19" s="2" t="n">
+      <c r="K19" s="3" t="n">
         <v>5076</v>
       </c>
     </row>
@@ -1077,28 +1089,28 @@
           <t>mediterranean_diet</t>
         </is>
       </c>
-      <c r="B20" s="2" t="n">
+      <c r="B20" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C20" s="3" t="n">
+      <c r="C20" s="4" t="n">
         <v>1.02</v>
       </c>
-      <c r="D20" s="3" t="n">
+      <c r="D20" s="4" t="n">
         <v>0.92</v>
       </c>
-      <c r="E20" s="3" t="n">
+      <c r="E20" s="4" t="n">
         <v>1.13</v>
       </c>
-      <c r="F20" s="3" t="inlineStr"/>
-      <c r="G20" s="3" t="inlineStr"/>
-      <c r="H20" s="4" t="n">
+      <c r="F20" s="4" t="inlineStr"/>
+      <c r="G20" s="4" t="inlineStr"/>
+      <c r="H20" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="I20" s="5" t="inlineStr"/>
-      <c r="J20" s="2" t="n">
+      <c r="I20" s="6" t="inlineStr"/>
+      <c r="J20" s="3" t="n">
         <v>106146</v>
       </c>
-      <c r="K20" s="2" t="inlineStr"/>
+      <c r="K20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1106,28 +1118,28 @@
           <t>butyric_acid</t>
         </is>
       </c>
-      <c r="B21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C21" s="3" t="n">
+      <c r="B21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" s="4" t="n">
         <v>1.08</v>
       </c>
-      <c r="D21" s="3" t="n">
+      <c r="D21" s="4" t="n">
         <v>1.01</v>
       </c>
-      <c r="E21" s="3" t="n">
+      <c r="E21" s="4" t="n">
         <v>1.15</v>
       </c>
-      <c r="F21" s="3" t="inlineStr"/>
-      <c r="G21" s="3" t="inlineStr"/>
-      <c r="H21" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" s="5" t="inlineStr"/>
-      <c r="J21" s="2" t="n">
+      <c r="F21" s="4" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr"/>
+      <c r="H21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="6" t="inlineStr"/>
+      <c r="J21" s="3" t="n">
         <v>142239</v>
       </c>
-      <c r="K21" s="2" t="inlineStr"/>
+      <c r="K21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1135,28 +1147,28 @@
           <t>eggs</t>
         </is>
       </c>
-      <c r="B22" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C22" s="3" t="n">
+      <c r="B22" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" s="4" t="n">
         <v>1.14</v>
       </c>
-      <c r="D22" s="3" t="n">
+      <c r="D22" s="4" t="n">
         <v>1.01</v>
       </c>
-      <c r="E22" s="3" t="n">
+      <c r="E22" s="4" t="n">
         <v>1.28</v>
       </c>
-      <c r="F22" s="3" t="inlineStr"/>
-      <c r="G22" s="3" t="inlineStr"/>
-      <c r="H22" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" s="5" t="inlineStr"/>
-      <c r="J22" s="2" t="n">
+      <c r="F22" s="4" t="inlineStr"/>
+      <c r="G22" s="4" t="inlineStr"/>
+      <c r="H22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="6" t="inlineStr"/>
+      <c r="J22" s="3" t="n">
         <v>842149</v>
       </c>
-      <c r="K22" s="2" t="n">
+      <c r="K22" s="3" t="n">
         <v>4924</v>
       </c>
     </row>
@@ -1166,28 +1178,28 @@
           <t>western_pattern_diet</t>
         </is>
       </c>
-      <c r="B23" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C23" s="3" t="n">
+      <c r="B23" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="4" t="n">
         <v>1.23</v>
       </c>
-      <c r="D23" s="3" t="n">
+      <c r="D23" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="E23" s="3" t="n">
+      <c r="E23" s="4" t="n">
         <v>1.84</v>
       </c>
-      <c r="F23" s="3" t="inlineStr"/>
-      <c r="G23" s="3" t="inlineStr"/>
-      <c r="H23" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="5" t="inlineStr"/>
-      <c r="J23" s="2" t="n">
+      <c r="F23" s="4" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr"/>
+      <c r="H23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="6" t="inlineStr"/>
+      <c r="J23" s="3" t="n">
         <v>43469</v>
       </c>
-      <c r="K23" s="2" t="inlineStr"/>
+      <c r="K23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1195,28 +1207,28 @@
           <t>plant_protein_intake</t>
         </is>
       </c>
-      <c r="B24" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C24" s="3" t="n">
+      <c r="B24" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" s="4" t="n">
         <v>1.24</v>
       </c>
-      <c r="D24" s="3" t="n">
+      <c r="D24" s="4" t="n">
         <v>1.04</v>
       </c>
-      <c r="E24" s="3" t="n">
+      <c r="E24" s="4" t="n">
         <v>1.47</v>
       </c>
-      <c r="F24" s="3" t="inlineStr"/>
-      <c r="G24" s="3" t="inlineStr"/>
-      <c r="H24" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" s="5" t="inlineStr"/>
-      <c r="J24" s="2" t="n">
+      <c r="F24" s="4" t="inlineStr"/>
+      <c r="G24" s="4" t="inlineStr"/>
+      <c r="H24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="6" t="inlineStr"/>
+      <c r="J24" s="3" t="n">
         <v>150671</v>
       </c>
-      <c r="K24" s="2" t="n">
+      <c r="K24" s="3" t="n">
         <v>2170</v>
       </c>
     </row>
@@ -1226,28 +1238,28 @@
           <t>multivitamin</t>
         </is>
       </c>
-      <c r="B25" s="2" t="n">
+      <c r="B25" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C25" s="3" t="n">
+      <c r="C25" s="4" t="n">
         <v>1.27</v>
       </c>
-      <c r="D25" s="3" t="n">
+      <c r="D25" s="4" t="n">
         <v>1.04</v>
       </c>
-      <c r="E25" s="3" t="n">
+      <c r="E25" s="4" t="n">
         <v>1.56</v>
       </c>
-      <c r="F25" s="3" t="inlineStr"/>
-      <c r="G25" s="3" t="inlineStr"/>
-      <c r="H25" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" s="5" t="inlineStr"/>
-      <c r="J25" s="2" t="n">
+      <c r="F25" s="4" t="inlineStr"/>
+      <c r="G25" s="4" t="inlineStr"/>
+      <c r="H25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="6" t="inlineStr"/>
+      <c r="J25" s="3" t="n">
         <v>343481</v>
       </c>
-      <c r="K25" s="2" t="n">
+      <c r="K25" s="3" t="n">
         <v>2040</v>
       </c>
     </row>
@@ -1257,34 +1269,34 @@
           <t>alcohol</t>
         </is>
       </c>
-      <c r="B26" s="2" t="n">
+      <c r="B26" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="C26" s="3" t="n">
+      <c r="C26" s="4" t="n">
         <v>1.28</v>
       </c>
-      <c r="D26" s="3" t="n">
+      <c r="D26" s="4" t="n">
         <v>0.73</v>
       </c>
-      <c r="E26" s="3" t="n">
+      <c r="E26" s="4" t="n">
         <v>2.26</v>
       </c>
-      <c r="F26" s="3" t="n">
+      <c r="F26" s="4" t="n">
         <v>0.11</v>
       </c>
-      <c r="G26" s="3" t="n">
+      <c r="G26" s="4" t="n">
         <v>15.55</v>
       </c>
-      <c r="H26" s="4" t="n">
+      <c r="H26" s="5" t="n">
         <v>80</v>
       </c>
-      <c r="I26" s="5" t="n">
+      <c r="I26" s="6" t="n">
         <v>0.4695295847551806</v>
       </c>
-      <c r="J26" s="2" t="n">
+      <c r="J26" s="3" t="n">
         <v>166503</v>
       </c>
-      <c r="K26" s="2" t="inlineStr"/>
+      <c r="K26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1292,28 +1304,28 @@
           <t>dairy</t>
         </is>
       </c>
-      <c r="B27" s="2" t="n">
+      <c r="B27" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C27" s="3" t="n">
+      <c r="C27" s="4" t="n">
         <v>1.39</v>
       </c>
-      <c r="D27" s="3" t="n">
+      <c r="D27" s="4" t="n">
         <v>1.08</v>
       </c>
-      <c r="E27" s="3" t="n">
+      <c r="E27" s="4" t="n">
         <v>1.78</v>
       </c>
-      <c r="F27" s="3" t="inlineStr"/>
-      <c r="G27" s="3" t="inlineStr"/>
-      <c r="H27" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I27" s="5" t="inlineStr"/>
-      <c r="J27" s="2" t="n">
+      <c r="F27" s="4" t="inlineStr"/>
+      <c r="G27" s="4" t="inlineStr"/>
+      <c r="H27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="6" t="inlineStr"/>
+      <c r="J27" s="3" t="n">
         <v>80266</v>
       </c>
-      <c r="K27" s="2" t="n">
+      <c r="K27" s="3" t="n">
         <v>439</v>
       </c>
     </row>
@@ -1323,34 +1335,34 @@
           <t>processed_meat_intake</t>
         </is>
       </c>
-      <c r="B28" s="2" t="n">
+      <c r="B28" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C28" s="3" t="n">
+      <c r="C28" s="4" t="n">
         <v>1.41</v>
       </c>
-      <c r="D28" s="3" t="n">
+      <c r="D28" s="4" t="n">
         <v>1.2</v>
       </c>
-      <c r="E28" s="3" t="n">
+      <c r="E28" s="4" t="n">
         <v>1.65</v>
       </c>
-      <c r="F28" s="3" t="n">
+      <c r="F28" s="4" t="n">
         <v>0.5</v>
       </c>
-      <c r="G28" s="3" t="n">
+      <c r="G28" s="4" t="n">
         <v>3.95</v>
       </c>
-      <c r="H28" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I28" s="5" t="n">
+      <c r="H28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="6" t="n">
         <v>0.1471089201375944</v>
       </c>
-      <c r="J28" s="2" t="n">
+      <c r="J28" s="3" t="n">
         <v>177383</v>
       </c>
-      <c r="K28" s="2" t="n">
+      <c r="K28" s="3" t="n">
         <v>2103</v>
       </c>
     </row>
@@ -1360,28 +1372,28 @@
           <t>genistein</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C29" s="3" t="n">
+      <c r="B29" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" s="4" t="n">
         <v>1.51</v>
       </c>
-      <c r="D29" s="3" t="n">
+      <c r="D29" s="4" t="n">
         <v>1.02</v>
       </c>
-      <c r="E29" s="3" t="n">
+      <c r="E29" s="4" t="n">
         <v>2.22</v>
       </c>
-      <c r="F29" s="3" t="inlineStr"/>
-      <c r="G29" s="3" t="inlineStr"/>
-      <c r="H29" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" s="5" t="inlineStr"/>
-      <c r="J29" s="2" t="n">
+      <c r="F29" s="4" t="inlineStr"/>
+      <c r="G29" s="4" t="inlineStr"/>
+      <c r="H29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="6" t="inlineStr"/>
+      <c r="J29" s="3" t="n">
         <v>27004</v>
       </c>
-      <c r="K29" s="2" t="n">
+      <c r="K29" s="3" t="n">
         <v>287</v>
       </c>
     </row>
@@ -1391,34 +1403,34 @@
           <t>calcium</t>
         </is>
       </c>
-      <c r="B30" s="2" t="n">
+      <c r="B30" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="C30" s="3" t="n">
+      <c r="C30" s="4" t="n">
         <v>1.53</v>
       </c>
-      <c r="D30" s="3" t="n">
+      <c r="D30" s="4" t="n">
         <v>0.98</v>
       </c>
-      <c r="E30" s="3" t="n">
+      <c r="E30" s="4" t="n">
         <v>2.38</v>
       </c>
-      <c r="F30" s="3" t="n">
+      <c r="F30" s="4" t="n">
         <v>0.36</v>
       </c>
-      <c r="G30" s="3" t="n">
+      <c r="G30" s="4" t="n">
         <v>6.44</v>
       </c>
-      <c r="H30" s="4" t="n">
+      <c r="H30" s="5" t="n">
         <v>76</v>
       </c>
-      <c r="I30" s="5" t="n">
-        <v>0.9970484632921826</v>
-      </c>
-      <c r="J30" s="2" t="n">
+      <c r="I30" s="6" t="n">
+        <v>0.9970484632921824</v>
+      </c>
+      <c r="J30" s="3" t="n">
         <v>98931</v>
       </c>
-      <c r="K30" s="2" t="inlineStr"/>
+      <c r="K30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1426,34 +1438,34 @@
           <t>red_meat</t>
         </is>
       </c>
-      <c r="B31" s="2" t="n">
+      <c r="B31" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="C31" s="3" t="n">
+      <c r="C31" s="4" t="n">
         <v>1.57</v>
       </c>
-      <c r="D31" s="3" t="n">
+      <c r="D31" s="4" t="n">
         <v>1.2</v>
       </c>
-      <c r="E31" s="3" t="n">
+      <c r="E31" s="4" t="n">
         <v>2.05</v>
       </c>
-      <c r="F31" s="3" t="n">
+      <c r="F31" s="4" t="n">
         <v>0.88</v>
       </c>
-      <c r="G31" s="3" t="n">
+      <c r="G31" s="4" t="n">
         <v>2.81</v>
       </c>
-      <c r="H31" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I31" s="5" t="n">
-        <v>0.2560168911966049</v>
-      </c>
-      <c r="J31" s="2" t="n">
+      <c r="H31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="6" t="n">
+        <v>0.2560168911966048</v>
+      </c>
+      <c r="J31" s="3" t="n">
         <v>101424</v>
       </c>
-      <c r="K31" s="2" t="n">
+      <c r="K31" s="3" t="n">
         <v>1376</v>
       </c>
     </row>
@@ -1463,28 +1475,28 @@
           <t>mineral_supplements</t>
         </is>
       </c>
-      <c r="B32" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C32" s="3" t="n">
+      <c r="B32" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" s="4" t="n">
         <v>1.8</v>
       </c>
-      <c r="D32" s="3" t="n">
+      <c r="D32" s="4" t="n">
         <v>1.19</v>
       </c>
-      <c r="E32" s="3" t="n">
+      <c r="E32" s="4" t="n">
         <v>2.73</v>
       </c>
-      <c r="F32" s="3" t="inlineStr"/>
-      <c r="G32" s="3" t="inlineStr"/>
-      <c r="H32" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I32" s="5" t="inlineStr"/>
-      <c r="J32" s="2" t="n">
+      <c r="F32" s="4" t="inlineStr"/>
+      <c r="G32" s="4" t="inlineStr"/>
+      <c r="H32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="6" t="inlineStr"/>
+      <c r="J32" s="3" t="n">
         <v>47240</v>
       </c>
-      <c r="K32" s="2" t="n">
+      <c r="K32" s="3" t="n">
         <v>1143</v>
       </c>
     </row>
@@ -1494,34 +1506,34 @@
           <t>alpha_linolenic_acid</t>
         </is>
       </c>
-      <c r="B33" s="2" t="n">
+      <c r="B33" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C33" s="3" t="n">
+      <c r="C33" s="4" t="n">
         <v>1.85</v>
       </c>
-      <c r="D33" s="3" t="n">
+      <c r="D33" s="4" t="n">
         <v>1.03</v>
       </c>
-      <c r="E33" s="3" t="n">
+      <c r="E33" s="4" t="n">
         <v>3.31</v>
       </c>
-      <c r="F33" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G33" s="3" t="n">
+      <c r="F33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="4" t="n">
         <v>2021.94</v>
       </c>
-      <c r="H33" s="4" t="n">
+      <c r="H33" s="5" t="n">
         <v>86</v>
       </c>
-      <c r="I33" s="5" t="n">
-        <v>0.01966497897827823</v>
-      </c>
-      <c r="J33" s="2" t="n">
+      <c r="I33" s="6" t="n">
+        <v>0.01966497897827825</v>
+      </c>
+      <c r="J33" s="3" t="n">
         <v>383989</v>
       </c>
-      <c r="K33" s="2" t="n">
+      <c r="K33" s="3" t="n">
         <v>3504</v>
       </c>
     </row>
@@ -1531,28 +1543,28 @@
           <t>betaine</t>
         </is>
       </c>
-      <c r="B34" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C34" s="3" t="n">
+      <c r="B34" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" s="4" t="n">
         <v>1.86</v>
       </c>
-      <c r="D34" s="3" t="n">
+      <c r="D34" s="4" t="n">
         <v>1.05</v>
       </c>
-      <c r="E34" s="3" t="n">
+      <c r="E34" s="4" t="n">
         <v>3.3</v>
       </c>
-      <c r="F34" s="3" t="inlineStr"/>
-      <c r="G34" s="3" t="inlineStr"/>
-      <c r="H34" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I34" s="5" t="inlineStr"/>
-      <c r="J34" s="2" t="n">
+      <c r="F34" s="4" t="inlineStr"/>
+      <c r="G34" s="4" t="inlineStr"/>
+      <c r="H34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="6" t="inlineStr"/>
+      <c r="J34" s="3" t="n">
         <v>692</v>
       </c>
-      <c r="K34" s="2" t="n">
+      <c r="K34" s="3" t="n">
         <v>173</v>
       </c>
     </row>
@@ -1562,28 +1574,28 @@
           <t>carnitine</t>
         </is>
       </c>
-      <c r="B35" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C35" s="3" t="n">
+      <c r="B35" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="D35" s="3" t="n">
+      <c r="D35" s="4" t="n">
         <v>1.13</v>
       </c>
-      <c r="E35" s="3" t="n">
+      <c r="E35" s="4" t="n">
         <v>3.56</v>
       </c>
-      <c r="F35" s="3" t="inlineStr"/>
-      <c r="G35" s="3" t="inlineStr"/>
-      <c r="H35" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I35" s="5" t="inlineStr"/>
-      <c r="J35" s="2" t="n">
+      <c r="F35" s="4" t="inlineStr"/>
+      <c r="G35" s="4" t="inlineStr"/>
+      <c r="H35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" s="6" t="inlineStr"/>
+      <c r="J35" s="3" t="n">
         <v>692</v>
       </c>
-      <c r="K35" s="2" t="n">
+      <c r="K35" s="3" t="n">
         <v>173</v>
       </c>
     </row>
@@ -1593,28 +1605,28 @@
           <t>choline</t>
         </is>
       </c>
-      <c r="B36" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C36" s="3" t="n">
+      <c r="B36" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" s="4" t="n">
         <v>2.19</v>
       </c>
-      <c r="D36" s="3" t="n">
+      <c r="D36" s="4" t="n">
         <v>1.23</v>
       </c>
-      <c r="E36" s="3" t="n">
+      <c r="E36" s="4" t="n">
         <v>3.9</v>
       </c>
-      <c r="F36" s="3" t="inlineStr"/>
-      <c r="G36" s="3" t="inlineStr"/>
-      <c r="H36" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I36" s="5" t="inlineStr"/>
-      <c r="J36" s="2" t="n">
+      <c r="F36" s="4" t="inlineStr"/>
+      <c r="G36" s="4" t="inlineStr"/>
+      <c r="H36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" s="6" t="inlineStr"/>
+      <c r="J36" s="3" t="n">
         <v>692</v>
       </c>
-      <c r="K36" s="2" t="n">
+      <c r="K36" s="3" t="n">
         <v>173</v>
       </c>
     </row>
@@ -1624,28 +1636,28 @@
           <t>monounsaturated_fat_mufa</t>
         </is>
       </c>
-      <c r="B37" s="2" t="n">
+      <c r="B37" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C37" s="3" t="n">
+      <c r="C37" s="4" t="n">
         <v>2.39</v>
       </c>
-      <c r="D37" s="3" t="n">
+      <c r="D37" s="4" t="n">
         <v>1.37</v>
       </c>
-      <c r="E37" s="3" t="n">
+      <c r="E37" s="4" t="n">
         <v>4.15</v>
       </c>
-      <c r="F37" s="3" t="inlineStr"/>
-      <c r="G37" s="3" t="inlineStr"/>
-      <c r="H37" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I37" s="5" t="inlineStr"/>
-      <c r="J37" s="2" t="n">
+      <c r="F37" s="4" t="inlineStr"/>
+      <c r="G37" s="4" t="inlineStr"/>
+      <c r="H37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" s="6" t="inlineStr"/>
+      <c r="J37" s="3" t="n">
         <v>2234</v>
       </c>
-      <c r="K37" s="2" t="inlineStr"/>
+      <c r="K37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1653,28 +1665,28 @@
           <t>polyunsaturated_fat_pufa</t>
         </is>
       </c>
-      <c r="B38" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C38" s="3" t="n">
+      <c r="B38" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" s="4" t="n">
         <v>2.7</v>
       </c>
-      <c r="D38" s="3" t="n">
+      <c r="D38" s="4" t="n">
         <v>1.1</v>
       </c>
-      <c r="E38" s="3" t="n">
+      <c r="E38" s="4" t="n">
         <v>6.8</v>
       </c>
-      <c r="F38" s="3" t="inlineStr"/>
-      <c r="G38" s="3" t="inlineStr"/>
-      <c r="H38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I38" s="5" t="inlineStr"/>
-      <c r="J38" s="2" t="n">
+      <c r="F38" s="4" t="inlineStr"/>
+      <c r="G38" s="4" t="inlineStr"/>
+      <c r="H38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="6" t="inlineStr"/>
+      <c r="J38" s="3" t="n">
         <v>1037</v>
       </c>
-      <c r="K38" s="2" t="inlineStr"/>
+      <c r="K38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1682,28 +1694,28 @@
           <t>omega_3_fatty_acids</t>
         </is>
       </c>
-      <c r="B39" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C39" s="3" t="n">
+      <c r="B39" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" s="4" t="n">
         <v>3.43</v>
       </c>
-      <c r="D39" s="3" t="n">
+      <c r="D39" s="4" t="n">
         <v>1.67</v>
       </c>
-      <c r="E39" s="3" t="n">
+      <c r="E39" s="4" t="n">
         <v>7.04</v>
       </c>
-      <c r="F39" s="3" t="inlineStr"/>
-      <c r="G39" s="3" t="inlineStr"/>
-      <c r="H39" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I39" s="5" t="inlineStr"/>
-      <c r="J39" s="2" t="n">
+      <c r="F39" s="4" t="inlineStr"/>
+      <c r="G39" s="4" t="inlineStr"/>
+      <c r="H39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="6" t="inlineStr"/>
+      <c r="J39" s="3" t="n">
         <v>47855</v>
       </c>
-      <c r="K39" s="2" t="n">
+      <c r="K39" s="3" t="n">
         <v>126</v>
       </c>
     </row>

</xml_diff>